<commit_message>
Update xlsx parser to improve material summary aggregation
- Modified scripts/xlsx_parser.py to implement new aggregation logic based on IFC class, Russian type name, and material, calculating counts, volumes, and areas according to material number groups (e.g., 02/03/31 as volume, 30 as area/volume depending on name)
- Updated .gitignore to include uploads/ directory and adjust environment/dependency ignore rules
- Replaced old materials_summary.json and materials_summary.xlsx output files reflecting the new aggregation format with columns Type (RU), Element Type, Material, Quantity (pcs), Volume (m³), Area (m²)
</commit_message>
<xml_diff>
--- a/uploads/21c3edf4-5bb2-4c20-9c9c-e3733e45913a/materials_summary.xlsx
+++ b/uploads/21c3edf4-5bb2-4c20-9c9c-e3733e45913a/materials_summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Сводка по материалам" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Сводка по элементам" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -433,111 +433,327 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="56" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>№</t>
+          <t>Тип (RU)</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Тип элемента</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Материал</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Группа</t>
-        </is>
-      </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Ед. изм.</t>
+          <t>Количество, шт</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Общее количество</t>
+          <t>Объем, м³</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Кол-во элементов</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Примеры элементов</t>
+          <t>Площадь, м²</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>1</v>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Арматурные_сетки</t>
+        </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
+          <t>IfcReinforcingMesh</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Не указан</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Колонны</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>IfcColumn</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
           <t>Бетон</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="D3" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>643698.583</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>1265682.415</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Лестницы</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>IfcStair</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>Бетон</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>шт</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="n">
-        <v>1352</v>
-      </c>
-      <c r="F2" s="2" t="n">
-        <v>1352</v>
-      </c>
-      <c r="G2" s="2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Неизвестный материал</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Другой</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>шт</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="n">
-        <v>1940</v>
-      </c>
-      <c r="F3" s="2" t="n">
-        <v>1940</v>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Жилой дом; -1_Подземный этаж_основной; 1_Этаж_основной</t>
-        </is>
+      <c r="D4" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Пандусы</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>IfcRamp</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Бетон</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Перекрытия</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>IfcSlab</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Бетон</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>119</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>2987992.324</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>44171.162</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Перекрытия</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>IfcSlab</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Не указан</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>8869.183000000001</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>5640.589</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Проемы</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>IfcOpeningElement</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Не указан</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>490</v>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Прочие_элементы</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>IfcBuildingElementProxy</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Не указан</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>1291</v>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Стены</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>IfcWall</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Бетон</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>1147</v>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>2363579.814</v>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>20253.419</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Стены</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>IfcWall</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Не указан</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>74</v>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>30568.661</v>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>2715.508</v>
       </c>
     </row>
   </sheetData>

</xml_diff>